<commit_message>
data: 2026-07-15 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-15.xlsx
+++ b/data/daily/2026-07/2026-07-15.xlsx
@@ -803,7 +803,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -811,29 +811,29 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2입 추가 증정 "선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 앰플 2입 추가 증정</t>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>61,900원</t>
+          <t>33,000원</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/4965835</t>
+          <t>https://gift.kakao.com/product/12860133</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -841,22 +841,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
+          <t>2입 추가 증정 "선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 앰플 2입 추가 증정</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>아일로</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>45,900원</t>
+          <t>61,900원</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11566779</t>
+          <t>https://gift.kakao.com/product/4965835</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -881,12 +881,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>33,000원</t>
+          <t>45,900원</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12860133</t>
+          <t>https://gift.kakao.com/product/11566779</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1127,7 +1127,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1135,29 +1135,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1165,29 +1165,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>루테인 30정 30일분</t>
+          <t>[김종국 PICK] 익스트림 아르기닌 에너지온 2개입 2일분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>1,500원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000126&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=987253277&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1195,29 +1195,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>[신혜선 PICK] 동국 마이팝 푸룬＆식이섬유</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911029&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>마그네슘</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1225,29 +1225,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>마그네슘 샷 25ml x 5병 5일분</t>
+          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000204&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1255,29 +1255,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rTG 오메가3 30캡슐 30일분</t>
+          <t>동화 부채표 편안활 5포 5일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000145&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=601618636&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>혈행</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1285,29 +1285,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>동국 맛있는 샐러드 미니볼 15포 15일분</t>
+          <t>코엔자임 Q10 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910891&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>녹차카테킨 30정 30일분</t>
+          <t>마그네슘 샷 25ml x 5병 5일분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1330,14 +1330,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000136&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000204&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1345,29 +1345,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>푸응 7days 팻버닝 21캡슐</t>
+          <t>마그네슘 30정 30일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>닥터블릿</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602085&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이지슬로 엑스트라버진 올리브오일＆레몬 4병</t>
+          <t>LG생활건강 이너뷰 진한 레드 석류 콜라겐 7포</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>자연관</t>
+          <t>이너뷰 바이 리튠</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1390,14 +1390,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032627034&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=994953529&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>비타민B 30정 30일분</t>
+          <t>rTG 오메가3 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1415,12 +1415,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000129&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000145&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1551,16 +1551,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>6.7</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1573,16 +1573,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>6.7</v>
+        <v>3.3</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -1639,16 +1639,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>23.3</v>
+        <v>26.7</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -1683,16 +1683,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>3.3</v>
+        <v>6.7</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -1705,16 +1705,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>23.3</v>
       </c>
       <c r="D12" t="n">
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>

</xml_diff>